<commit_message>
PCAs, phylotree, germination analysis and matrices updated, removal of 4 species no germination
</commit_message>
<xml_diff>
--- a/results/Traits PCA exploration.xlsx
+++ b/results/Traits PCA exploration.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17835"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17835" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Med_alltraits" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="67">
   <si>
     <t>Contributions</t>
   </si>
@@ -208,22 +208,28 @@
     <t>Saxifraga conifera</t>
   </si>
   <si>
-    <t>8 traits 21 species (without NAs)</t>
-  </si>
-  <si>
     <t>11 traits 19 species (without Nas)</t>
   </si>
   <si>
     <t>11 traits 23 species (with some Nas in leaves traits and BODMC)</t>
   </si>
   <si>
-    <t>8 traits 26 species (without NAs)</t>
-  </si>
-  <si>
-    <t>5 traits 21 species (without NAs)</t>
-  </si>
-  <si>
-    <t>5 traits 26 species (without NAs)</t>
+    <t>5 traits 18 species (without NAs)</t>
+  </si>
+  <si>
+    <t>8 traits 18 species (without NAs)</t>
+  </si>
+  <si>
+    <t>8 traits 25 species (without NAs)</t>
+  </si>
+  <si>
+    <t>5 traits 25 species (without NAs)</t>
+  </si>
+  <si>
+    <t>odds_C_WP od</t>
+  </si>
+  <si>
+    <t>ds_D_constant</t>
   </si>
 </sst>
 </file>
@@ -428,196 +434,6 @@
         <a:xfrm>
           <a:off x="12696825" y="1905000"/>
           <a:ext cx="8134350" cy="5019675"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>29248</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9401175" y="2476500"/>
-          <a:ext cx="9630448" cy="7772400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>664349</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>111900</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>638174</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>122677</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8789174" y="492900"/>
-          <a:ext cx="9117825" cy="9154777"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>561975</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>483381</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>145403</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5600700" y="0"/>
-          <a:ext cx="7541406" cy="7193903"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>692925</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>616725</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5484000" y="38100"/>
-          <a:ext cx="7543800" cy="7191375"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -910,10 +726,10 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" t="s">
         <v>60</v>
-      </c>
-      <c r="J1" t="s">
-        <v>61</v>
       </c>
       <c r="Q1" t="s">
         <v>44</v>
@@ -3425,7 +3241,7 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D1" t="s">
         <v>44</v>
@@ -3463,23 +3279,23 @@
       <c r="N3" s="13"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="9">
-        <v>16.689441777999999</v>
+        <v>18.985688</v>
       </c>
       <c r="C4" s="7">
-        <v>6.8771563999999996</v>
+        <v>1.6334010000000001</v>
       </c>
       <c r="D4" s="7">
-        <v>0.69988790000000001</v>
+        <v>0.17227870000000001</v>
       </c>
       <c r="E4" s="7">
-        <v>10.167385299999999</v>
+        <v>12.230522300000001</v>
       </c>
       <c r="F4" s="7">
-        <v>21.351747</v>
+        <v>17.12856</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -3492,23 +3308,23 @@
       <c r="O4" s="6"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="7">
-        <v>13.380522778</v>
+        <v>10.404294999999999</v>
       </c>
       <c r="C5" s="7">
-        <v>1.3102289</v>
+        <v>1.614981</v>
       </c>
       <c r="D5" s="11">
-        <v>21.681553699999998</v>
+        <v>41.377450000000003</v>
       </c>
       <c r="E5" s="7">
-        <v>26.91741699</v>
+        <v>11.347933299999999</v>
       </c>
       <c r="F5" s="7">
-        <v>10.014347000000001</v>
+        <v>10.933892</v>
       </c>
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
@@ -3521,23 +3337,23 @@
       <c r="O5" s="6"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="9">
-        <v>23.865445865000002</v>
+      <c r="A6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="7">
+        <v>14.74173</v>
       </c>
       <c r="C6" s="7">
-        <v>1.4155055999999999</v>
+        <v>6.2553380000000001</v>
       </c>
       <c r="D6" s="7">
-        <v>0.4414014</v>
+        <v>11.14279</v>
       </c>
       <c r="E6" s="7">
-        <v>2.0775585599999999</v>
+        <v>24.952536899999998</v>
       </c>
       <c r="F6" s="7">
-        <v>26.977423999999999</v>
+        <v>4.8151780000000004</v>
       </c>
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
@@ -3551,22 +3367,22 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B7" s="7">
-        <v>9.3106739390000008</v>
-      </c>
-      <c r="C7" s="7">
-        <v>24.203319</v>
+        <v>4.947044</v>
+      </c>
+      <c r="C7" s="10">
+        <v>37.788679999999999</v>
       </c>
       <c r="D7" s="7">
-        <v>6.2873625999999998</v>
+        <v>5.2075930000000001</v>
       </c>
       <c r="E7" s="7">
-        <v>5.1097289999999997E-2</v>
+        <v>4.2107416000000004</v>
       </c>
       <c r="F7" s="7">
-        <v>13.219109</v>
+        <v>9.4748950000000001</v>
       </c>
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
@@ -3579,23 +3395,23 @@
       <c r="O7" s="6"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>13</v>
+      <c r="A8" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="B8" s="7">
-        <v>7.4744809999999998E-3</v>
-      </c>
-      <c r="C8" s="10">
-        <v>27.1365765</v>
-      </c>
-      <c r="D8" s="11">
-        <v>41.206966100000002</v>
+        <v>15.491374</v>
+      </c>
+      <c r="C8" s="7">
+        <v>1.1648890000000001</v>
+      </c>
+      <c r="D8" s="7">
+        <v>3.7982749999999998</v>
       </c>
       <c r="E8" s="7">
-        <v>2.5004038</v>
+        <v>33.211504599999998</v>
       </c>
       <c r="F8" s="7">
-        <v>6.8461740000000004</v>
+        <v>3.609229</v>
       </c>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
@@ -3609,22 +3425,22 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="7">
-        <v>14.89513387</v>
+        <v>11</v>
+      </c>
+      <c r="B9" s="9">
+        <v>23.744232</v>
       </c>
       <c r="C9" s="7">
-        <v>6.9360837999999996</v>
+        <v>1.157705</v>
       </c>
       <c r="D9" s="7">
-        <v>5.1288115999999997</v>
+        <v>4.1810079999999997E-4</v>
       </c>
       <c r="E9" s="7">
-        <v>31.58498616</v>
+        <v>1.3513728</v>
       </c>
       <c r="F9" s="7">
-        <v>6.1774440000000004</v>
+        <v>29.315358</v>
       </c>
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
@@ -3637,23 +3453,23 @@
       <c r="O9" s="6"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>16</v>
+      <c r="A10" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="B10" s="7">
-        <v>6.925903924</v>
-      </c>
-      <c r="C10" s="10">
-        <v>31.8856267</v>
+        <v>10.432245999999999</v>
+      </c>
+      <c r="C10" s="7">
+        <v>20.763566000000001</v>
       </c>
       <c r="D10" s="7">
-        <v>7.5171692999999999</v>
+        <v>8.1982189999999999</v>
       </c>
       <c r="E10" s="7">
-        <v>1.0101356100000001</v>
+        <v>0.3686026</v>
       </c>
       <c r="F10" s="7">
-        <v>11.862721000000001</v>
+        <v>21.726469999999999</v>
       </c>
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
@@ -3667,22 +3483,22 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B11" s="7">
-        <v>14.925403364999999</v>
-      </c>
-      <c r="C11" s="7">
-        <v>0.23550309999999999</v>
-      </c>
-      <c r="D11" s="7">
-        <v>17.0368475</v>
+        <v>1.2533909999999999</v>
+      </c>
+      <c r="C11" s="10">
+        <v>29.62144</v>
+      </c>
+      <c r="D11" s="11">
+        <v>30.102979999999999</v>
       </c>
       <c r="E11" s="7">
-        <v>25.691016279999999</v>
+        <v>12.3267858</v>
       </c>
       <c r="F11" s="7">
-        <v>3.5510329999999999</v>
+        <v>2.9964179999999998</v>
       </c>
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
@@ -3725,13 +3541,13 @@
         <v>21</v>
       </c>
       <c r="B16" s="6">
-        <v>3.0447521000000002</v>
+        <v>3.0856205999999999</v>
       </c>
       <c r="C16" s="6">
-        <v>38.059401000000001</v>
+        <v>38.570256999999998</v>
       </c>
       <c r="D16" s="6">
-        <v>38.059399999999997</v>
+        <v>38.570259999999998</v>
       </c>
       <c r="J16" s="4"/>
     </row>
@@ -3740,13 +3556,13 @@
         <v>22</v>
       </c>
       <c r="B17" s="6">
-        <v>1.5877870999999999</v>
+        <v>1.5110895</v>
       </c>
       <c r="C17" s="6">
-        <v>19.847339000000002</v>
+        <v>18.888618999999998</v>
       </c>
       <c r="D17" s="6">
-        <v>57.906739999999999</v>
+        <v>57.458880000000001</v>
       </c>
       <c r="J17" s="4"/>
     </row>
@@ -3755,13 +3571,13 @@
         <v>23</v>
       </c>
       <c r="B18" s="6">
-        <v>1.0872731</v>
+        <v>1.0751807</v>
       </c>
       <c r="C18" s="6">
-        <v>13.590913</v>
+        <v>13.439759</v>
       </c>
       <c r="D18" s="6">
-        <v>71.497649999999993</v>
+        <v>70.89864</v>
       </c>
       <c r="J18" s="4"/>
     </row>
@@ -3770,13 +3586,13 @@
         <v>24</v>
       </c>
       <c r="B19" s="6">
-        <v>0.84637280000000004</v>
+        <v>0.90345900000000001</v>
       </c>
       <c r="C19" s="6">
-        <v>10.579660000000001</v>
+        <v>11.293238000000001</v>
       </c>
       <c r="D19" s="6">
-        <v>82.077309999999997</v>
+        <v>82.191869999999994</v>
       </c>
       <c r="J19" s="4"/>
     </row>
@@ -3785,13 +3601,13 @@
         <v>25</v>
       </c>
       <c r="B20" s="6">
-        <v>0.58190419999999998</v>
+        <v>0.62688080000000002</v>
       </c>
       <c r="C20" s="6">
-        <v>7.2738019999999999</v>
+        <v>7.8360089999999998</v>
       </c>
       <c r="D20" s="6">
-        <v>89.351119999999995</v>
+        <v>90.027879999999996</v>
       </c>
       <c r="J20" s="4"/>
     </row>
@@ -3800,13 +3616,13 @@
         <v>26</v>
       </c>
       <c r="B21" s="6">
-        <v>0.40108159999999998</v>
+        <v>0.36990980000000001</v>
       </c>
       <c r="C21" s="6">
-        <v>5.0135199999999998</v>
+        <v>4.6238720000000004</v>
       </c>
       <c r="D21" s="6">
-        <v>94.364639999999994</v>
+        <v>94.651759999999996</v>
       </c>
       <c r="J21" s="4"/>
     </row>
@@ -3815,13 +3631,13 @@
         <v>27</v>
       </c>
       <c r="B22" s="6">
-        <v>0.29642069999999998</v>
+        <v>0.30769479999999999</v>
       </c>
       <c r="C22" s="6">
-        <v>3.7052589999999999</v>
+        <v>3.8461850000000002</v>
       </c>
       <c r="D22" s="6">
-        <v>98.069890000000001</v>
+        <v>98.49794</v>
       </c>
       <c r="J22" s="4"/>
     </row>
@@ -3830,10 +3646,10 @@
         <v>28</v>
       </c>
       <c r="B23" s="6">
-        <v>0.1544084</v>
+        <v>0.1201648</v>
       </c>
       <c r="C23" s="6">
-        <v>1.930105</v>
+        <v>1.50206</v>
       </c>
       <c r="D23" s="6">
         <v>100</v>
@@ -3864,22 +3680,22 @@
         <v>9</v>
       </c>
       <c r="D28" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="H28" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="I28" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="J28" s="6"/>
       <c r="L28" s="4"/>
@@ -3892,25 +3708,25 @@
         <v>1</v>
       </c>
       <c r="C29" s="6">
-        <v>0.26276670000000002</v>
+        <v>0.26795829999999998</v>
       </c>
       <c r="D29" s="6">
-        <v>0.56828800000000002</v>
+        <v>-0.47614240000000002</v>
       </c>
       <c r="E29" s="6">
-        <v>0.52863468000000002</v>
+        <v>-0.15420990000000001</v>
       </c>
       <c r="F29" s="6">
-        <v>-5.2319049999999999E-2</v>
+        <v>-0.37218329999999999</v>
       </c>
       <c r="G29" s="6">
-        <v>-0.37034265999999999</v>
+        <v>0.57011480000000003</v>
       </c>
       <c r="H29" s="16">
-        <v>-0.1003709</v>
+        <v>0.52707930000000003</v>
       </c>
       <c r="I29" s="16">
-        <v>-0.34011750000000002</v>
+        <v>-9.5374509999999996E-2</v>
       </c>
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
@@ -3921,28 +3737,28 @@
         <v>9</v>
       </c>
       <c r="B30" s="6">
-        <v>0.26276674</v>
+        <v>0.26795834000000002</v>
       </c>
       <c r="C30" s="6">
         <v>1</v>
       </c>
       <c r="D30" s="6">
-        <v>0.54706250000000001</v>
+        <v>-0.10094473</v>
       </c>
       <c r="E30" s="6">
-        <v>0.29941484000000002</v>
+        <v>-0.2064156</v>
       </c>
       <c r="F30" s="6">
-        <v>0.26789096000000001</v>
+        <v>-0.3693613</v>
       </c>
       <c r="G30" s="6">
-        <v>-0.17365380999999999</v>
+        <v>0.50795429999999997</v>
       </c>
       <c r="H30" s="16">
-        <v>-0.25691580000000003</v>
+        <v>0.30780010000000002</v>
       </c>
       <c r="I30" s="16">
-        <v>-0.37544539999999998</v>
+        <v>0.18760525</v>
       </c>
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
@@ -3950,31 +3766,31 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B31" s="6">
-        <v>0.56828798999999997</v>
+        <v>-0.47614240000000002</v>
       </c>
       <c r="C31" s="6">
-        <v>0.54706250000000001</v>
+        <v>-0.1009447</v>
       </c>
       <c r="D31" s="6">
         <v>1</v>
       </c>
       <c r="E31" s="6">
-        <v>0.43479972</v>
+        <v>0.42013620000000002</v>
       </c>
       <c r="F31" s="6">
-        <v>-8.1268699999999999E-2</v>
+        <v>0.31530380000000002</v>
       </c>
       <c r="G31" s="6">
-        <v>-0.59107807000000001</v>
+        <v>-0.62100390000000005</v>
       </c>
       <c r="H31" s="16">
-        <v>-0.17137859999999999</v>
+        <v>-0.13254199999999999</v>
       </c>
       <c r="I31" s="16">
-        <v>-0.41787990000000003</v>
+        <v>-1.978181E-2</v>
       </c>
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
@@ -3982,31 +3798,31 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B32" s="6">
-        <v>0.52863468000000002</v>
+        <v>-0.15420991000000001</v>
       </c>
       <c r="C32" s="6">
-        <v>0.29941479999999998</v>
+        <v>-0.2064156</v>
       </c>
       <c r="D32" s="6">
-        <v>0.43479970000000001</v>
+        <v>0.42013616999999998</v>
       </c>
       <c r="E32" s="6">
         <v>1</v>
       </c>
       <c r="F32" s="6">
-        <v>-0.17792442999999999</v>
+        <v>0.43488290000000002</v>
       </c>
       <c r="G32" s="6">
-        <v>-9.7240919999999995E-2</v>
+        <v>-0.1312933</v>
       </c>
       <c r="H32" s="16">
-        <v>0.13598830000000001</v>
+        <v>0.13706589999999999</v>
       </c>
       <c r="I32" s="16">
-        <v>-0.2221525</v>
+        <v>-0.19716935999999999</v>
       </c>
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
@@ -4014,31 +3830,31 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B33" s="6">
-        <v>-5.2319049999999999E-2</v>
+        <v>-0.37218333999999997</v>
       </c>
       <c r="C33" s="6">
-        <v>0.26789099999999999</v>
+        <v>-0.3693613</v>
       </c>
       <c r="D33" s="6">
-        <v>-8.1268699999999999E-2</v>
+        <v>0.31530377999999998</v>
       </c>
       <c r="E33" s="6">
-        <v>-0.17792442999999999</v>
+        <v>0.43488290000000002</v>
       </c>
       <c r="F33" s="6">
         <v>1</v>
       </c>
       <c r="G33" s="6">
-        <v>-0.11480425</v>
+        <v>-0.4427835</v>
       </c>
       <c r="H33" s="16">
-        <v>-0.2549498</v>
+        <v>-0.24464910000000001</v>
       </c>
       <c r="I33" s="16">
-        <v>0.19763220000000001</v>
+        <v>0.24121381</v>
       </c>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
@@ -4046,31 +3862,31 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B34" s="6">
-        <v>-0.37034265999999999</v>
+        <v>0.57011478000000004</v>
       </c>
       <c r="C34" s="6">
-        <v>-0.1736538</v>
+        <v>0.50795429999999997</v>
       </c>
       <c r="D34" s="6">
-        <v>-0.59107810000000005</v>
+        <v>-0.62100387000000001</v>
       </c>
       <c r="E34" s="6">
-        <v>-9.7240919999999995E-2</v>
+        <v>-0.1312933</v>
       </c>
       <c r="F34" s="6">
-        <v>-0.11480425</v>
+        <v>-0.4427835</v>
       </c>
       <c r="G34" s="6">
         <v>1</v>
       </c>
       <c r="H34" s="16">
-        <v>0.48603089999999999</v>
+        <v>0.41058070000000002</v>
       </c>
       <c r="I34" s="16">
-        <v>0.32875959999999999</v>
+        <v>-0.26349139999999999</v>
       </c>
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
@@ -4078,31 +3894,31 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B35" s="6">
-        <v>-0.10037087</v>
+        <v>0.52707926000000005</v>
       </c>
       <c r="C35" s="6">
-        <v>-0.25691580000000003</v>
+        <v>0.30780010000000002</v>
       </c>
       <c r="D35" s="6">
-        <v>-0.17137859999999999</v>
+        <v>-0.13254198</v>
       </c>
       <c r="E35" s="6">
-        <v>0.13598832</v>
+        <v>0.13706589999999999</v>
       </c>
       <c r="F35" s="6">
-        <v>-0.25494977000000002</v>
+        <v>-0.24464910000000001</v>
       </c>
       <c r="G35" s="6">
-        <v>0.48603094000000002</v>
+        <v>0.41058070000000002</v>
       </c>
       <c r="H35" s="16">
         <v>1</v>
       </c>
       <c r="I35" s="16">
-        <v>0.44294699999999998</v>
+        <v>-0.24944298000000001</v>
       </c>
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
@@ -4110,28 +3926,28 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B36" s="6">
-        <v>-0.34011751000000001</v>
+        <v>-9.5374509999999996E-2</v>
       </c>
       <c r="C36" s="6">
-        <v>-0.37544539999999998</v>
+        <v>0.1876053</v>
       </c>
       <c r="D36" s="6">
-        <v>-0.41787990000000003</v>
+        <v>-1.978181E-2</v>
       </c>
       <c r="E36" s="6">
-        <v>-0.22215255</v>
+        <v>-0.19716939999999999</v>
       </c>
       <c r="F36" s="6">
-        <v>0.19763217999999999</v>
+        <v>0.24121380000000001</v>
       </c>
       <c r="G36" s="6">
-        <v>0.32875958999999999</v>
+        <v>-0.26349139999999999</v>
       </c>
       <c r="H36" s="16">
-        <v>0.44294699999999998</v>
+        <v>-0.249443</v>
       </c>
       <c r="I36" s="16">
         <v>1</v>
@@ -4175,7 +3991,6 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4189,7 +4004,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -4220,159 +4035,159 @@
         <v>32</v>
       </c>
       <c r="B4" s="7">
-        <v>13.408659</v>
+        <v>12.965892999999999</v>
       </c>
       <c r="C4" s="7">
-        <v>0.14828748</v>
+        <v>2.307346E-2</v>
       </c>
       <c r="D4" s="7">
-        <v>0.32828299999999999</v>
+        <v>1.166314053</v>
       </c>
       <c r="E4" s="7">
-        <v>43.717234869999999</v>
+        <v>39.774089519999997</v>
       </c>
       <c r="F4" s="7">
-        <v>41.044559999999997</v>
+        <v>44.7807569</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="9">
-        <v>29.335946</v>
+        <v>27.209951</v>
       </c>
       <c r="C5" s="7">
-        <v>1.330304E-2</v>
+        <v>0.14656937</v>
       </c>
       <c r="D5" s="7">
-        <v>0.1076145</v>
+        <v>3.9781529999999999E-3</v>
       </c>
       <c r="E5" s="7">
-        <v>8.0944226690000001</v>
+        <v>10.343790500000001</v>
       </c>
       <c r="F5" s="7">
-        <v>1.5478209999999999</v>
+        <v>1.2354947999999999</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="9">
-        <v>30.985916</v>
+      <c r="A6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="7">
+        <v>1.907775</v>
       </c>
       <c r="C6" s="7">
-        <v>3.78940659</v>
-      </c>
-      <c r="D6" s="7">
-        <v>2.9940323000000002</v>
+        <v>21.086691819999999</v>
+      </c>
+      <c r="D6" s="11">
+        <v>35.233238026999999</v>
       </c>
       <c r="E6" s="7">
-        <v>4.843048E-3</v>
+        <v>0.10749776</v>
       </c>
       <c r="F6" s="7">
-        <v>14.652526</v>
+        <v>0.99657519999999999</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="7">
+        <v>1.9495260000000001</v>
+      </c>
+      <c r="C7" s="10">
+        <v>31.575072339999998</v>
+      </c>
+      <c r="D7" s="7">
+        <v>13.707763475</v>
+      </c>
+      <c r="E7" s="7">
+        <v>3.26862349</v>
+      </c>
+      <c r="F7" s="7">
+        <v>5.6274693999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="7">
+        <v>4.7364519999999999</v>
+      </c>
+      <c r="C8" s="10">
+        <v>41.219700099999997</v>
+      </c>
+      <c r="D8" s="7">
+        <v>7.4153611999999994E-2</v>
+      </c>
+      <c r="E8" s="7">
+        <v>0.66942966999999998</v>
+      </c>
+      <c r="F8" s="7">
+        <v>5.7225178000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="9">
+        <v>28.927278000000001</v>
+      </c>
+      <c r="C9" s="7">
+        <v>5.3885635199999999</v>
+      </c>
+      <c r="D9" s="7">
+        <v>3.219572919</v>
+      </c>
+      <c r="E9" s="7">
+        <v>2.675251E-2</v>
+      </c>
+      <c r="F9" s="7">
+        <v>16.193429999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="7">
-        <v>15.258298999999999</v>
-      </c>
-      <c r="C7" s="7">
-        <v>4.111948E-2</v>
-      </c>
-      <c r="D7" s="7">
-        <v>9.5578550999999994</v>
-      </c>
-      <c r="E7" s="7">
-        <v>26.423521405999999</v>
-      </c>
-      <c r="F7" s="7">
-        <v>6.5805150000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="B10" s="7">
+        <v>14.977034</v>
+      </c>
+      <c r="C10" s="7">
+        <v>1.8520559999999998E-2</v>
+      </c>
+      <c r="D10" s="7">
+        <v>8.1464683250000007</v>
+      </c>
+      <c r="E10" s="7">
+        <v>27.7805331</v>
+      </c>
+      <c r="F10" s="7">
+        <v>10.0472328</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="7">
-        <v>2.306559</v>
-      </c>
-      <c r="C8" s="7">
-        <v>0.30931449</v>
-      </c>
-      <c r="D8" s="11">
-        <v>46.715651100000002</v>
-      </c>
-      <c r="E8" s="7">
-        <v>17.318413216</v>
-      </c>
-      <c r="F8" s="7">
-        <v>17.533985999999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="7">
-        <v>2.3739599999999998</v>
-      </c>
-      <c r="C9" s="7">
-        <v>26.729057359999999</v>
-      </c>
-      <c r="D9" s="11">
-        <v>23.4138071</v>
-      </c>
-      <c r="E9" s="7">
-        <v>7.9713152999999995E-2</v>
-      </c>
-      <c r="F9" s="7">
-        <v>2.7961109999999998</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="7">
-        <v>2.6501160000000001</v>
-      </c>
-      <c r="C10" s="10">
-        <v>27.81555809</v>
-      </c>
-      <c r="D10" s="7">
-        <v>16.258378700000002</v>
-      </c>
-      <c r="E10" s="7">
-        <v>3.3494040900000002</v>
-      </c>
-      <c r="F10" s="7">
-        <v>8.0537240000000008</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="B11" s="7">
-        <v>3.680545</v>
-      </c>
-      <c r="C11" s="10">
-        <v>41.153953479999998</v>
-      </c>
-      <c r="D11" s="7">
-        <v>0.62437819999999999</v>
+        <v>7.3260899999999998</v>
+      </c>
+      <c r="C11" s="7">
+        <v>0.54180883000000002</v>
+      </c>
+      <c r="D11" s="11">
+        <v>38.448511435</v>
       </c>
       <c r="E11" s="7">
-        <v>1.012447549</v>
+        <v>18.029283450000001</v>
       </c>
       <c r="F11" s="7">
-        <v>7.7907570000000002</v>
+        <v>15.3965231</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -4424,13 +4239,13 @@
         <v>21</v>
       </c>
       <c r="B18" s="6">
-        <v>2.1933064999999998</v>
+        <v>2.2657688500000002</v>
       </c>
       <c r="C18" s="6">
-        <v>27.416331</v>
+        <v>28.322111</v>
       </c>
       <c r="D18" s="6">
-        <v>27.416329999999999</v>
+        <v>28.322109999999999</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -4438,13 +4253,13 @@
         <v>22</v>
       </c>
       <c r="B19" s="6">
-        <v>1.8806769000000001</v>
+        <v>1.89479084</v>
       </c>
       <c r="C19" s="6">
-        <v>23.508461</v>
+        <v>23.684885999999999</v>
       </c>
       <c r="D19" s="6">
-        <v>50.924790000000002</v>
+        <v>52.006999999999998</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -4452,13 +4267,13 @@
         <v>23</v>
       </c>
       <c r="B20" s="6">
-        <v>1.3277736</v>
+        <v>1.3007536099999999</v>
       </c>
       <c r="C20" s="6">
-        <v>16.597169999999998</v>
+        <v>16.259419999999999</v>
       </c>
       <c r="D20" s="6">
-        <v>67.521960000000007</v>
+        <v>68.266419999999997</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -4466,13 +4281,13 @@
         <v>24</v>
       </c>
       <c r="B21" s="6">
-        <v>0.91848099999999999</v>
+        <v>0.92367385000000002</v>
       </c>
       <c r="C21" s="6">
-        <v>11.481013000000001</v>
+        <v>11.545923</v>
       </c>
       <c r="D21" s="6">
-        <v>79.002970000000005</v>
+        <v>79.812340000000006</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -4480,13 +4295,13 @@
         <v>25</v>
       </c>
       <c r="B22" s="6">
-        <v>0.71096420000000005</v>
+        <v>0.71543917999999995</v>
       </c>
       <c r="C22" s="6">
-        <v>8.8870520000000006</v>
+        <v>8.94299</v>
       </c>
       <c r="D22" s="6">
-        <v>87.890029999999996</v>
+        <v>88.755330000000001</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -4494,13 +4309,13 @@
         <v>26</v>
       </c>
       <c r="B23" s="6">
-        <v>0.58939739999999996</v>
+        <v>0.57873770999999996</v>
       </c>
       <c r="C23" s="6">
-        <v>7.3674670000000004</v>
+        <v>7.2342209999999998</v>
       </c>
       <c r="D23" s="6">
-        <v>95.257490000000004</v>
+        <v>95.989549999999994</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -4508,13 +4323,13 @@
         <v>27</v>
       </c>
       <c r="B24" s="6">
-        <v>0.26068550000000001</v>
+        <v>0.22345957</v>
       </c>
       <c r="C24" s="6">
-        <v>3.258569</v>
+        <v>2.7932450000000002</v>
       </c>
       <c r="D24" s="6">
-        <v>98.516059999999996</v>
+        <v>98.782799999999995</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -4522,10 +4337,10 @@
         <v>28</v>
       </c>
       <c r="B25" s="6">
-        <v>0.118715</v>
+        <v>9.7376389999999993E-2</v>
       </c>
       <c r="C25" s="6">
-        <v>1.483938</v>
+        <v>1.2172050000000001</v>
       </c>
       <c r="D25" s="6">
         <v>100</v>
@@ -4563,22 +4378,22 @@
         <v>9</v>
       </c>
       <c r="D30" t="s">
+        <v>15</v>
+      </c>
+      <c r="E30" t="s">
+        <v>65</v>
+      </c>
+      <c r="F30" t="s">
+        <v>66</v>
+      </c>
+      <c r="G30" t="s">
         <v>11</v>
       </c>
-      <c r="E30" t="s">
+      <c r="H30" t="s">
         <v>12</v>
       </c>
-      <c r="F30" t="s">
+      <c r="I30" t="s">
         <v>13</v>
-      </c>
-      <c r="G30" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -4589,25 +4404,25 @@
         <v>1</v>
       </c>
       <c r="C31" s="6">
-        <v>0.27818614000000003</v>
+        <v>0.27490462999999998</v>
       </c>
       <c r="D31" s="6">
-        <v>0.27439384</v>
+        <v>-0.13476752</v>
       </c>
       <c r="E31" s="6">
-        <v>0.12304482999999999</v>
+        <v>0.13753862</v>
       </c>
       <c r="F31" s="6">
-        <v>0.12390548999999999</v>
+        <v>-0.13989862</v>
       </c>
       <c r="G31" s="6">
-        <v>-0.13982633</v>
+        <v>0.26863015000000001</v>
       </c>
       <c r="H31" s="6">
-        <v>0.11500128</v>
+        <v>0.12654625999999999</v>
       </c>
       <c r="I31" s="6">
-        <v>-0.13761888999999999</v>
+        <v>0.1871765</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4615,199 +4430,199 @@
         <v>9</v>
       </c>
       <c r="B32" s="6">
-        <v>0.27818609999999999</v>
+        <v>0.2749046</v>
       </c>
       <c r="C32" s="6">
         <v>1</v>
       </c>
       <c r="D32" s="6">
-        <v>0.60122553999999995</v>
+        <v>-8.390562E-2</v>
       </c>
       <c r="E32" s="6">
-        <v>0.40254010000000001</v>
+        <v>3.8792779999999999E-2</v>
       </c>
       <c r="F32" s="6">
-        <v>7.3084109999999994E-2</v>
+        <v>-0.12338151999999999</v>
       </c>
       <c r="G32" s="6">
-        <v>-8.6650249999999998E-2</v>
+        <v>0.59989174999999995</v>
       </c>
       <c r="H32" s="6">
-        <v>2.8329590000000002E-2</v>
+        <v>0.40462728999999997</v>
       </c>
       <c r="I32" s="6">
-        <v>-0.12242469</v>
+        <v>0.14106389999999999</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B33" s="6">
-        <v>0.27439380000000002</v>
+        <v>-0.13476750000000001</v>
       </c>
       <c r="C33" s="6">
-        <v>0.60122553999999995</v>
+        <v>-8.390562E-2</v>
       </c>
       <c r="D33" s="6">
         <v>1</v>
       </c>
       <c r="E33" s="6">
-        <v>0.29845155000000001</v>
+        <v>9.5953849999999993E-2</v>
       </c>
       <c r="F33" s="6">
-        <v>0.11229899</v>
+        <v>0.61605745999999995</v>
       </c>
       <c r="G33" s="6">
-        <v>-8.7635480000000002E-2</v>
+        <v>-8.3271629999999999E-2</v>
       </c>
       <c r="H33" s="6">
-        <v>0.47806009999999999</v>
+        <v>3.7818909999999997E-2</v>
       </c>
       <c r="I33" s="6">
-        <v>-6.8670460000000003E-2</v>
+        <v>0.25231189999999998</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B34" s="6">
-        <v>0.1230448</v>
+        <v>0.13753860000000001</v>
       </c>
       <c r="C34" s="6">
-        <v>0.40254010000000001</v>
+        <v>3.8792779999999999E-2</v>
       </c>
       <c r="D34" s="6">
-        <v>0.29845155000000001</v>
+        <v>9.5953849999999993E-2</v>
       </c>
       <c r="E34" s="6">
         <v>1</v>
       </c>
       <c r="F34" s="6">
-        <v>0.16880118</v>
+        <v>0.52006156999999997</v>
       </c>
       <c r="G34" s="6">
-        <v>3.9430319999999998E-2</v>
+        <v>0.50457618999999998</v>
       </c>
       <c r="H34" s="6">
-        <v>-1.1101969999999999E-2</v>
+        <v>-1.6895899999999998E-2</v>
       </c>
       <c r="I34" s="6">
-        <v>-9.9861409999999998E-2</v>
+        <v>-0.1161341</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B35" s="6">
-        <v>0.1239055</v>
+        <v>-0.13989860000000001</v>
       </c>
       <c r="C35" s="6">
-        <v>7.3084109999999994E-2</v>
+        <v>-0.12338151999999999</v>
       </c>
       <c r="D35" s="6">
-        <v>0.11229899</v>
+        <v>0.61605745999999995</v>
       </c>
       <c r="E35" s="6">
-        <v>0.16880118</v>
+        <v>0.52006156999999997</v>
       </c>
       <c r="F35" s="6">
         <v>1</v>
       </c>
       <c r="G35" s="6">
-        <v>0.31771063999999999</v>
+        <v>-7.015557E-2</v>
       </c>
       <c r="H35" s="6">
-        <v>-7.5132019999999994E-2</v>
+        <v>-9.9469210000000002E-2</v>
       </c>
       <c r="I35" s="6">
-        <v>-0.1512162</v>
+        <v>-0.26613789999999998</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B36" s="6">
-        <v>-0.13982629999999999</v>
+        <v>0.26863009999999998</v>
       </c>
       <c r="C36" s="6">
-        <v>-8.6650249999999998E-2</v>
+        <v>0.59989174999999995</v>
       </c>
       <c r="D36" s="6">
-        <v>-8.7635480000000002E-2</v>
+        <v>-8.3271629999999999E-2</v>
       </c>
       <c r="E36" s="6">
-        <v>3.9430319999999998E-2</v>
+        <v>0.50457618999999998</v>
       </c>
       <c r="F36" s="6">
-        <v>0.31771063999999999</v>
+        <v>-7.015557E-2</v>
       </c>
       <c r="G36" s="6">
         <v>1</v>
       </c>
       <c r="H36" s="6">
-        <v>0.10555196999999999</v>
+        <v>0.30179117</v>
       </c>
       <c r="I36" s="6">
-        <v>0.61393527000000003</v>
+        <v>0.2110176</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B37" s="6">
-        <v>0.1150013</v>
+        <v>0.1265463</v>
       </c>
       <c r="C37" s="6">
-        <v>2.8329590000000002E-2</v>
+        <v>0.40462728999999997</v>
       </c>
       <c r="D37" s="6">
-        <v>0.47806009999999999</v>
+        <v>3.7818909999999997E-2</v>
       </c>
       <c r="E37" s="6">
-        <v>-1.1101969999999999E-2</v>
+        <v>-1.6895899999999998E-2</v>
       </c>
       <c r="F37" s="6">
-        <v>-7.5132019999999994E-2</v>
+        <v>-9.9469210000000002E-2</v>
       </c>
       <c r="G37" s="6">
-        <v>0.10555196999999999</v>
+        <v>0.30179117</v>
       </c>
       <c r="H37" s="6">
         <v>1</v>
       </c>
       <c r="I37" s="6">
-        <v>0.50715504</v>
+        <v>0.21000150000000001</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B38" s="6">
-        <v>-0.13761889999999999</v>
+        <v>0.1871765</v>
       </c>
       <c r="C38" s="6">
-        <v>-0.12242469</v>
+        <v>0.14106387000000001</v>
       </c>
       <c r="D38" s="6">
-        <v>-6.8670460000000003E-2</v>
+        <v>0.25231186</v>
       </c>
       <c r="E38" s="6">
-        <v>-9.9861409999999998E-2</v>
+        <v>-0.11613407000000001</v>
       </c>
       <c r="F38" s="6">
-        <v>-0.1512162</v>
+        <v>-0.26613785000000001</v>
       </c>
       <c r="G38" s="6">
-        <v>0.61393527000000003</v>
+        <v>0.21101755999999999</v>
       </c>
       <c r="H38" s="6">
-        <v>0.50715504</v>
+        <v>0.21000152999999999</v>
       </c>
       <c r="I38" s="6">
         <v>1</v>
@@ -4827,7 +4642,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4843,7 +4657,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D1" t="s">
         <v>44</v>
@@ -4873,63 +4687,63 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="18">
-        <v>26.5862403</v>
+        <v>26.560912999999999</v>
       </c>
       <c r="C4" s="5">
-        <v>2.2427151599999999</v>
+        <v>2.4148969999999999E-2</v>
       </c>
       <c r="D4" s="5">
-        <v>27.41995</v>
+        <v>27.013010000000001</v>
       </c>
       <c r="E4" s="5">
-        <v>22.75291</v>
+        <v>26.014709499999999</v>
       </c>
       <c r="F4" s="5">
-        <v>20.998189</v>
+        <v>20.387221</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="5">
-        <v>18.663889099999999</v>
+        <v>15.703687</v>
       </c>
       <c r="C5" s="19">
-        <v>24.925225959999999</v>
+        <v>32.460217299999996</v>
       </c>
       <c r="D5" s="5">
-        <v>23.541889999999999</v>
+        <v>20.733059999999998</v>
       </c>
       <c r="E5" s="5">
-        <v>7.058052</v>
+        <v>10.3752616</v>
       </c>
       <c r="F5" s="5">
-        <v>25.810943000000002</v>
+        <v>20.727777</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="18">
-        <v>30.985259299999999</v>
+        <v>30.333687999999999</v>
       </c>
       <c r="C6" s="5">
-        <v>8.9057910000000004E-2</v>
+        <v>1.259011E-2</v>
       </c>
       <c r="D6" s="5">
-        <v>12.691660000000001</v>
+        <v>16.144290000000002</v>
       </c>
       <c r="E6" s="5">
-        <v>16.404710000000001</v>
+        <v>15.7693248</v>
       </c>
       <c r="F6" s="5">
-        <v>39.82931</v>
+        <v>37.740105</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -4937,39 +4751,39 @@
         <v>12</v>
       </c>
       <c r="B7" s="5">
-        <v>23.660830700000002</v>
+        <v>24.179449000000002</v>
       </c>
       <c r="C7" s="5">
-        <v>7.02930514</v>
+        <v>2.6030436099999998</v>
       </c>
       <c r="D7" s="5">
-        <v>10.079750000000001</v>
+        <v>18.208169999999999</v>
       </c>
       <c r="E7" s="5">
-        <v>53.783410000000003</v>
+        <v>46.940184500000001</v>
       </c>
       <c r="F7" s="5">
-        <v>5.446701</v>
+        <v>8.0691559999999996</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="5">
-        <v>0.1037806</v>
+        <v>3.2222629999999999</v>
       </c>
       <c r="C8" s="19">
-        <v>65.713695830000006</v>
+        <v>64.900000009999999</v>
       </c>
       <c r="D8" s="5">
-        <v>26.266749999999998</v>
+        <v>17.901479999999999</v>
       </c>
       <c r="E8" s="5">
-        <v>9.1675389999999995E-4</v>
+        <v>0.90051959999999998</v>
       </c>
       <c r="F8" s="5">
-        <v>7.9148569999999996</v>
+        <v>13.075741000000001</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -4999,13 +4813,13 @@
         <v>21</v>
       </c>
       <c r="B14" s="6">
-        <v>2.3356385999999998</v>
+        <v>2.3514134000000002</v>
       </c>
       <c r="C14" s="6">
-        <v>46.712772000000001</v>
+        <v>47.028269999999999</v>
       </c>
       <c r="D14" s="6">
-        <v>46.712769999999999</v>
+        <v>47.028269999999999</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -5013,13 +4827,13 @@
         <v>22</v>
       </c>
       <c r="B15" s="6">
-        <v>1.2298526000000001</v>
+        <v>1.1808038999999999</v>
       </c>
       <c r="C15" s="6">
-        <v>24.597052999999999</v>
+        <v>23.61608</v>
       </c>
       <c r="D15" s="6">
-        <v>71.309830000000005</v>
+        <v>70.644350000000003</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -5027,13 +4841,13 @@
         <v>23</v>
       </c>
       <c r="B16" s="6">
-        <v>0.63920120000000002</v>
+        <v>0.67959809999999998</v>
       </c>
       <c r="C16" s="6">
-        <v>12.784025</v>
+        <v>13.59196</v>
       </c>
       <c r="D16" s="6">
-        <v>84.093850000000003</v>
+        <v>84.236310000000003</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -5041,13 +4855,13 @@
         <v>24</v>
       </c>
       <c r="B17" s="6">
-        <v>0.52376440000000002</v>
+        <v>0.54889759999999999</v>
       </c>
       <c r="C17" s="6">
-        <v>10.475288000000001</v>
+        <v>10.97795</v>
       </c>
       <c r="D17" s="6">
-        <v>94.569140000000004</v>
+        <v>95.214259999999996</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -5055,10 +4869,10 @@
         <v>25</v>
       </c>
       <c r="B18" s="6">
-        <v>0.27154309999999998</v>
+        <v>0.239287</v>
       </c>
       <c r="C18" s="6">
-        <v>5.4308620000000003</v>
+        <v>4.7857399999999997</v>
       </c>
       <c r="D18" s="6">
         <v>100</v>
@@ -5095,16 +4909,16 @@
         <v>1</v>
       </c>
       <c r="C23" s="6">
-        <v>0.26276670000000002</v>
+        <v>0.26795829999999998</v>
       </c>
       <c r="D23" s="6">
-        <v>0.56828800000000002</v>
+        <v>0.57011480000000003</v>
       </c>
       <c r="E23" s="6">
-        <v>0.52863470000000001</v>
+        <v>0.52707930000000003</v>
       </c>
       <c r="F23" s="6">
-        <v>-5.2319049999999999E-2</v>
+        <v>-9.5374509999999996E-2</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -5112,19 +4926,19 @@
         <v>9</v>
       </c>
       <c r="B24" s="6">
-        <v>0.26276674</v>
+        <v>0.26795834000000002</v>
       </c>
       <c r="C24" s="6">
         <v>1</v>
       </c>
       <c r="D24" s="6">
-        <v>0.54706250000000001</v>
+        <v>0.50795429999999997</v>
       </c>
       <c r="E24" s="6">
-        <v>0.29941479999999998</v>
+        <v>0.30780010000000002</v>
       </c>
       <c r="F24" s="6">
-        <v>0.26789096000000001</v>
+        <v>0.18760525</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -5132,19 +4946,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="6">
-        <v>0.56828798999999997</v>
+        <v>0.57011478000000004</v>
       </c>
       <c r="C25" s="6">
-        <v>0.54706250000000001</v>
+        <v>0.50795429999999997</v>
       </c>
       <c r="D25" s="6">
         <v>1</v>
       </c>
       <c r="E25" s="6">
-        <v>0.43479970000000001</v>
+        <v>0.41058070000000002</v>
       </c>
       <c r="F25" s="6">
-        <v>-8.1268699999999999E-2</v>
+        <v>-0.26349139999999999</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -5152,19 +4966,19 @@
         <v>12</v>
       </c>
       <c r="B26" s="6">
-        <v>0.52863468000000002</v>
+        <v>0.52707926000000005</v>
       </c>
       <c r="C26" s="6">
-        <v>0.29941479999999998</v>
+        <v>0.30780010000000002</v>
       </c>
       <c r="D26" s="6">
-        <v>0.43479970000000001</v>
+        <v>0.41058070000000002</v>
       </c>
       <c r="E26" s="6">
         <v>1</v>
       </c>
       <c r="F26" s="6">
-        <v>-0.17792442999999999</v>
+        <v>-0.24944298000000001</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -5172,16 +4986,16 @@
         <v>13</v>
       </c>
       <c r="B27" s="6">
-        <v>-5.2319049999999999E-2</v>
+        <v>-9.5374509999999996E-2</v>
       </c>
       <c r="C27" s="6">
-        <v>0.26789099999999999</v>
+        <v>0.1876053</v>
       </c>
       <c r="D27" s="6">
-        <v>-8.1268699999999999E-2</v>
+        <v>-0.26349139999999999</v>
       </c>
       <c r="E27" s="6">
-        <v>-0.17792440000000001</v>
+        <v>-0.249443</v>
       </c>
       <c r="F27" s="6">
         <v>1</v>
@@ -5206,7 +5020,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5247,107 +5061,107 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="14">
-        <v>12.996131</v>
+        <v>12.567506</v>
       </c>
       <c r="C4" s="14">
-        <v>0.49676789999999998</v>
+        <v>17.413620000000002</v>
       </c>
       <c r="D4" s="20">
-        <v>67.600264229999993</v>
+        <v>49.651454600000001</v>
       </c>
       <c r="E4" s="14">
-        <v>18.790661</v>
+        <v>20.120231</v>
       </c>
       <c r="F4" s="14">
-        <v>0.1161751</v>
+        <v>0.24718799999999999</v>
       </c>
       <c r="G4" s="13"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="18">
-        <v>33.085949999999997</v>
+        <v>30.672536000000001</v>
       </c>
       <c r="C5" s="14">
-        <v>6.6186813000000004</v>
+        <v>12.211845</v>
       </c>
       <c r="D5" s="14">
-        <v>0.93696994</v>
+        <v>0.66283289999999995</v>
       </c>
       <c r="E5" s="14">
-        <v>3.7758129999999999</v>
+        <v>2.5315479999999999</v>
       </c>
       <c r="F5" s="14">
-        <v>55.5825855</v>
+        <v>53.921238000000002</v>
       </c>
       <c r="G5" s="13"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="18">
-        <v>30.481366999999999</v>
+        <v>29.094726999999999</v>
       </c>
       <c r="C6" s="14">
-        <v>4.6467155</v>
+        <v>4.6358240000000004</v>
       </c>
       <c r="D6" s="14">
-        <v>2.3136150000000001E-2</v>
+        <v>1.647751</v>
       </c>
       <c r="E6" s="14">
-        <v>25.243886</v>
+        <v>24.762712000000001</v>
       </c>
       <c r="F6" s="14">
-        <v>39.604894899999998</v>
+        <v>39.858986000000002</v>
       </c>
       <c r="G6" s="13"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="14">
-        <v>19.218067999999999</v>
+        <v>18.500167000000001</v>
       </c>
       <c r="C7" s="14">
-        <v>1.3052501999999999</v>
+        <v>3.2524039999999999</v>
       </c>
       <c r="D7" s="20">
-        <v>31.411842719999999</v>
+        <v>29.9080932</v>
       </c>
       <c r="E7" s="14">
-        <v>44.127268000000001</v>
+        <v>44.108597000000003</v>
       </c>
       <c r="F7" s="14">
-        <v>3.9375713999999999</v>
+        <v>4.2307379999999997</v>
       </c>
       <c r="G7" s="13"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="14">
-        <v>4.2184840000000001</v>
+        <v>9.165063</v>
       </c>
       <c r="C8" s="19">
-        <v>86.932585099999997</v>
+        <v>62.486306999999996</v>
       </c>
       <c r="D8" s="14">
-        <v>2.7786970000000001E-2</v>
+        <v>18.129868399999999</v>
       </c>
       <c r="E8" s="14">
-        <v>8.0623710000000006</v>
+        <v>8.4769109999999994</v>
       </c>
       <c r="F8" s="14">
-        <v>0.75877320000000004</v>
+        <v>1.7418499999999999</v>
       </c>
       <c r="G8" s="13"/>
     </row>
@@ -5378,13 +5192,13 @@
         <v>21</v>
       </c>
       <c r="B14" s="6">
-        <v>2.0843123000000001</v>
+        <v>2.1515803999999998</v>
       </c>
       <c r="C14" s="6">
-        <v>41.686245999999997</v>
+        <v>43.031607999999999</v>
       </c>
       <c r="D14" s="6">
-        <v>41.686250000000001</v>
+        <v>43.031610000000001</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -5392,13 +5206,13 @@
         <v>22</v>
       </c>
       <c r="B15" s="6">
-        <v>0.9839213</v>
+        <v>0.93106230000000001</v>
       </c>
       <c r="C15" s="6">
-        <v>19.678425000000001</v>
+        <v>18.621247</v>
       </c>
       <c r="D15" s="6">
-        <v>61.364669999999997</v>
+        <v>61.652850000000001</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -5406,13 +5220,13 @@
         <v>23</v>
       </c>
       <c r="B16" s="6">
-        <v>0.88593759999999999</v>
+        <v>0.86937929999999997</v>
       </c>
       <c r="C16" s="6">
-        <v>17.718751000000001</v>
+        <v>17.387585000000001</v>
       </c>
       <c r="D16" s="6">
-        <v>79.083420000000004</v>
+        <v>79.040440000000004</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -5420,13 +5234,13 @@
         <v>24</v>
       </c>
       <c r="B17" s="6">
-        <v>0.66465600000000002</v>
+        <v>0.67034729999999998</v>
       </c>
       <c r="C17" s="6">
-        <v>13.29312</v>
+        <v>13.406946</v>
       </c>
       <c r="D17" s="6">
-        <v>92.376540000000006</v>
+        <v>92.447389999999999</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -5434,10 +5248,10 @@
         <v>25</v>
       </c>
       <c r="B18" s="6">
-        <v>0.38117279999999998</v>
+        <v>0.37763069999999999</v>
       </c>
       <c r="C18" s="6">
-        <v>7.6234570000000001</v>
+        <v>7.5526140000000002</v>
       </c>
       <c r="D18" s="6">
         <v>100</v>
@@ -5474,16 +5288,16 @@
         <v>1</v>
       </c>
       <c r="C23" s="6">
-        <v>0.27818614000000003</v>
+        <v>0.2749046</v>
       </c>
       <c r="D23" s="6">
-        <v>0.27439380000000002</v>
+        <v>0.26863009999999998</v>
       </c>
       <c r="E23" s="6">
-        <v>0.1230448</v>
+        <v>0.1265463</v>
       </c>
       <c r="F23" s="6">
-        <v>0.12390548999999999</v>
+        <v>0.1871765</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -5491,19 +5305,19 @@
         <v>9</v>
       </c>
       <c r="B24" s="6">
-        <v>0.27818609999999999</v>
+        <v>0.2749046</v>
       </c>
       <c r="C24" s="6">
         <v>1</v>
       </c>
       <c r="D24" s="6">
-        <v>0.60122549999999997</v>
+        <v>0.59989179999999998</v>
       </c>
       <c r="E24" s="6">
-        <v>0.40254010000000001</v>
+        <v>0.40462730000000002</v>
       </c>
       <c r="F24" s="6">
-        <v>7.3084109999999994E-2</v>
+        <v>0.14106389999999999</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -5511,19 +5325,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="6">
-        <v>0.27439380000000002</v>
+        <v>0.26863009999999998</v>
       </c>
       <c r="C25" s="6">
-        <v>0.60122553999999995</v>
+        <v>0.59989179999999998</v>
       </c>
       <c r="D25" s="6">
         <v>1</v>
       </c>
       <c r="E25" s="6">
-        <v>0.29845159999999998</v>
+        <v>0.30179119999999998</v>
       </c>
       <c r="F25" s="6">
-        <v>0.11229899</v>
+        <v>0.2110176</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -5531,19 +5345,19 @@
         <v>12</v>
       </c>
       <c r="B26" s="6">
-        <v>0.1230448</v>
+        <v>0.1265463</v>
       </c>
       <c r="C26" s="6">
-        <v>0.40254010000000001</v>
+        <v>0.40462730000000002</v>
       </c>
       <c r="D26" s="6">
-        <v>0.29845159999999998</v>
+        <v>0.30179119999999998</v>
       </c>
       <c r="E26" s="6">
         <v>1</v>
       </c>
       <c r="F26" s="6">
-        <v>0.16880118</v>
+        <v>0.21000150000000001</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -5551,16 +5365,16 @@
         <v>13</v>
       </c>
       <c r="B27" s="6">
-        <v>0.1239055</v>
+        <v>0.1871765</v>
       </c>
       <c r="C27" s="6">
-        <v>7.3084109999999994E-2</v>
+        <v>0.14106389999999999</v>
       </c>
       <c r="D27" s="6">
-        <v>0.112299</v>
+        <v>0.2110176</v>
       </c>
       <c r="E27" s="6">
-        <v>0.16880120000000001</v>
+        <v>0.21000150000000001</v>
       </c>
       <c r="F27" s="6">
         <v>1</v>
@@ -5585,6 +5399,5 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>